<commit_message>
maybe I should delete this
</commit_message>
<xml_diff>
--- a/w9-extractor.xlsx
+++ b/w9-extractor.xlsx
@@ -74,12 +74,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -447,7 +450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -505,12 +508,12 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ralpha THat LLC</t>
+          <t>Palitree Inc LLC</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>That LLC</t>
+          <t>Palitree LLC</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -520,17 +523,147 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>TEst, Houston 77077</t>
+          <t>111 City Boulivard St</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>TEst, Houston 77077</t>
+          <t>Maryland, OK</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Jines INC</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Samuel Jines</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>C Corporation</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>222 City Boulivard St</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>England, DC</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>477-44-1774</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>12-2172214</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Ralpha THat LLC</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>That LLC</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>C Corporation</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>1221 Saint INC</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>TEst, Houston 77077 a</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>712-13-3333</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>90-2000081</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Ralpha THat LLC</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>That LLC</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>C Corporation</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1221 Saint INC</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>TEst, Houston 77077</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>122-43-3331</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+      <c r="H5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="inlineStr"/>
+      <c r="H7" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update W-9 extraction logic, add OCR fallback and test harness
</commit_message>
<xml_diff>
--- a/w9-extractor.xlsx
+++ b/w9-extractor.xlsx
@@ -531,8 +531,16 @@
           <t>Maryland, OK</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>111-14-5396</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>10-0126120</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr"/>
     </row>
     <row r="3" ht="18" customHeight="1">
@@ -601,12 +609,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>712-13-3333</t>
+          <t>121-33-3335</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>90-2000081</t>
+          <t>07-1626210</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -639,7 +647,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>122-43-3331</t>
+          <t>111-33-3333</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr"/>

</xml_diff>